<commit_message>
Update Bao Hai Phong category URL from sub-folder to root /phap-luat in config.py
</commit_message>
<xml_diff>
--- a/storage/reports/Bao_Cao_Rui_Ro_2026-07-28_den_2026-07-28.xlsx
+++ b/storage/reports/Bao_Cao_Rui_Ro_2026-07-28_den_2026-07-28.xlsx
@@ -504,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -524,7 +524,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Khoảng thời gian: 2026-07-28 đến 2026-07-28 | Khu vực: Tất cả 6 tỉnh | Tổng số rủi ro: 53</t>
+          <t>Khoảng thời gian: 2026-07-28 đến 2026-07-28 | Khu vực: Tất cả 6 tỉnh | Tổng số rủi ro: 62</t>
         </is>
       </c>
     </row>
@@ -559,12 +559,12 @@
     <row r="5" ht="55" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>H.N.A</t>
+          <t>Công ty TNHH Toàn Mỹ liên quan những sai phạm xảy ra năm 2019; Công ty TNHH Toàn Mỹ được cơ quan; Công ty Toàn Mỹ; Ông Tạ Viết Đông; Bị can Tạ Viết Đông</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Lực lượng công an thành phố Hải Phòng phát hiện và xử lý nhiều nhóm thanh thiếu niên vi phạm trật tự an toàn giao thông, mang theo hung khí như kiếm dài, dao, tuýp sắt để gây rối trật tự công cộng. Trong 6 tháng đầu năm 2026, cơ quan điều tra đã khởi tố 23 vụ với 215 bị can liên quan đến tội phạm đường phố.</t>
+          <t>Theo cơ quan điều tra, ông Tạ Viết Đông bị bắt vì chỉ đạo phá dỡ cầu tàu của doanh nghiệp khi chưa thanh toán theo thỏa thuận và chưa có quyết định cưỡng chế.. Ngày 20/7, Văn phòng Cơ quan Cảnh sát điều tra Công an TP Hải Phòng cho biết đã bắt tạm giam ông Tạ Viết Đông (còn gọi là Tạ Tòng Đông, nguyên Giám đốc Ban Quản lý dự án) để điều tra về t...</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -574,12 +574,12 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Khởi tố/Gây rối trật tự công cộng</t>
+          <t>khởi tố, tạm giam, bị can</t>
         </is>
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25
+          <t>2026-07-28
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -587,12 +587,12 @@
     <row r="6" ht="55" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>Thuế cơ sở 11</t>
+          <t>Công ty TNHH Toàn Mỹ; Công ty TNHH Toàn Mỹ được cơ quan; Công ty CP Tập đoàn Đầu tư thương mại Quang Hưng</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Viện Kiểm sát nhân dân khu vực 12 (Hải Phòng) có văn bản kiến nghị Thuế cơ sở 11 khắc phục việc chậm thực hiện nghĩa vụ thuế liên quan đến giao đất tái định cư, gây ảnh hưởng đến quyền lợi của một công dân cao tuổi.</t>
+          <t>Nguyên Giám đốc Ban Quản lý Dự án đầu tư xây dựng phát triển đô thị thành phố Hải Phòng Tạ Tòng Đông bị bắt tạm giam để điều tra về tội lạm quyền trong khi thi hành công vụ.. Theo thông tin từ Cổng thông tin điện tử Công an thành phố Hải Phòng, Văn phòng Cơ quan Cảnh sát điều tra Công an thành phố đã khởi tố bị can và thi hành lệnh bắt tạm giam ...</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
@@ -602,12 +602,12 @@
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>Chậm thực hiện nghĩa vụ thuế</t>
+          <t>khởi tố, tạm giam, lừa đảo</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25
+          <t>2026-07-28
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -615,27 +615,27 @@
     <row r="7" ht="55" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Vũ Thị Thảo</t>
+          <t>Công ty MediUSA</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Công an quận Lê Chân (Hải Phòng) triệt phá đường dây vận chuyển trái phép chất ma túy qua dịch vụ chuyển phát nhanh, bắt giữ 3 đối tượng gồm Vũ Thị Thảo, Nguyễn Kim Hùng và Đặng Quang Chính, thu giữ 20 gam Methamphetamine.</t>
+          <t>TAND Hà Nội xét xử vụ án sản xuất 88 dòng thực phẩm chức năng giả liên quan đến cựu CEO Nguyễn Năng Mạnh của Công ty MediUSA. Hai cựu cán bộ thuộc Cục Giám sát quản lý về Hải quan bị truy tố tội Nhận hối lộ vì đã nhận 1,5 tỷ đồng để giúp công ty này thông quan trái phép lô nguyên liệu trị giá 20 tỷ đồng.</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Hải Phòng</t>
+          <t>Hà Nội</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Khởi tố/Bắt tạm giam</t>
+          <t>Nhận hối lộ/Sản xuất hàng giả</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>2026-03-27
+          <t>2026-07-28
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -643,27 +643,27 @@
     <row r="8" ht="55" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>Công ty CP Tập đoàn Đầu tư thương mại Quang Hưng</t>
+          <t>Nguyễn Văn Mong</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Công an thành phố Hải Phòng đang xác minh nguồn tin về tội phạm đối với vụ việc có dấu hiệu lừa đảo chiếm đoạt tài sản liên quan đến Lưu Quang Hưng, Giám đốc Công ty CP Tập đoàn Đầu tư thương mại Quang Hưng trong các giao dịch mua bán căn hộ và đất đai.</t>
+          <t>Tòa án nhân dân tỉnh Bắc Ninh tuyên phạt bị cáo Nguyễn Văn Mong tổng mức án 18 năm tù về tội mua bán trái phép chất ma túy với vai trò cầm đầu ổ nhóm bán lẻ. Các đồng phạm khác cũng bị tuyên án từ 5 năm 6 tháng đến 8 năm 6 tháng tù.</t>
         </is>
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>Hải Phòng</t>
+          <t>Bắc Ninh</t>
         </is>
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>Điều tra tội phạm/Lừa đảo</t>
+          <t>Khởi tố/Bắt tạm giam</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>2026-07-26
+          <t>2026-07-28
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -671,27 +671,27 @@
     <row r="9" ht="55" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Chưa xác định</t>
+          <t>Hứa Văn Xương</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Công an thành phố Hải Phòng đã kịp thời ngăn chặn hai nhóm thanh thiếu niên mang theo hung khí chuẩn bị hỗn chiến và bàn giao các đối tượng liên quan để xử lý về hành vi trộm cắp tài sản.</t>
+          <t>Lực lượng chức năng phối hợp bắt quả tang đối tượng Hứa Văn Xương đang vận chuyển trái phép 30.000 viên ma túy tổng hợp (khối lượng gần 2,8kg) qua khu vực trạm thu phí cầu Thái Hà thuộc tỉnh Hưng Yên.</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Hải Phòng</t>
+          <t>Hưng Yên</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Gây rối trật tự công cộng/Trộm cắp</t>
+          <t>Vận chuyển trái phép chất ma túy</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>2026-07-27
+          <t>2026-07-28
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -699,27 +699,27 @@
     <row r="10" ht="55" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>Phạm Văn Chiến</t>
+          <t>Lê Quang Trường</t>
         </is>
       </c>
       <c r="B10" s="8" t="inlineStr">
         <is>
-          <t>Phòng Cảnh sát hình sự Công an thành phố Hải Phòng đã bắt giữ đối tượng Phạm Văn Chiến, nghi phạm dùng hung khí sát hại một phụ nữ tại phường Lưu Kiếm do mâu thuẫn ghen tuông tình ái.</t>
+          <t>Lê Quang Trường đã xin đi nhờ xe máy, sau đó đánh chủ xe, cướp phương tiện mang đi cầm cố lấy 3 triệu đồng tiêu xài cá nhân và đã bị bắt giữ.</t>
         </is>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Hải Phòng</t>
+          <t>Đắk Lắk</t>
         </is>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>Khởi tố/Bắt tạm giam</t>
+          <t>Cướp tài sản</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25
+          <t>2026-07-28
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -732,7 +732,7 @@
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Bão số 2 hoạt động trên Biển Đông có khả năng mạnh lên cấp 12, gây gió mạnh, sóng lớn trên biển và mưa lớn diện rộng cho khu vực Bắc Bộ và Nam Bộ, đe dọa an toàn hàng hải và nguy cơ ngập úng, sạt lở đất.</t>
+          <t>Bài viết kể lại vụ án hình sự đối với bị cáo G. phạm tội 'Cố ý gây thương tích' trong một xô xát tại công trình xây dựng, sau đó đã được tòa án xét xử sơ thẩm và phúc thẩm tuyên án treo nhờ sự trợ giúp pháp lý.</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -742,12 +742,12 @@
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Thiên tai/Bão lũ</t>
+          <t>Khởi tố/Xét xử hình sự</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25
+          <t>2026-07-27
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -755,22 +755,22 @@
     <row r="12" ht="55" customHeight="1">
       <c r="A12" s="8" t="inlineStr">
         <is>
-          <t>Công an xã Thượng Cốc</t>
+          <t>Chưa xác định</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Công an xã Thượng Cốc đã xử phạt hành chính nhiều trường hợp vi phạm trật tự an toàn giao thông và vi phạm tại các cơ sở kinh doanh có điều kiện, đồng thời phát hiện 3 trường hợp dương tính với ma túy qua kiểm tra nhanh.</t>
+          <t>Tỉnh Quảng Ninh phê bình một số địa phương có tỷ lệ tiêm phòng vắc-xin cho đàn gia súc, gia cầm đạt thấp dưới 50%, tiềm ẩn nguy cơ bùng phát dịch bệnh nguy hiểm trên diện rộng và gây ô nhiễm môi trường.</t>
         </is>
       </c>
       <c r="C12" s="9" t="inlineStr">
         <is>
-          <t>Phú Thọ</t>
+          <t>Quảng Ninh</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>Xử phạt hành chính/Vi phạm trật tự an toàn</t>
+          <t>Vi phạm quy định thú y</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
@@ -783,22 +783,22 @@
     <row r="13" ht="55" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Chưa xác định</t>
+          <t>Công an xã Thượng Cốc</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Tỉnh Quảng Ninh phê bình một số địa phương có tỷ lệ tiêm phòng vắc-xin cho đàn gia súc, gia cầm đạt thấp dưới 50%, tiềm ẩn nguy cơ bùng phát dịch bệnh nguy hiểm trên diện rộng và gây ô nhiễm môi trường.</t>
+          <t>Công an xã Thượng Cốc đã xử phạt hành chính nhiều trường hợp vi phạm trật tự an toàn giao thông và vi phạm tại các cơ sở kinh doanh có điều kiện, đồng thời phát hiện 3 trường hợp dương tính với ma túy qua kiểm tra nhanh.</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Quảng Ninh</t>
+          <t>Phú Thọ</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Vi phạm quy định thú y</t>
+          <t>Xử phạt hành chính/Vi phạm trật tự an toàn</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
@@ -816,17 +816,17 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Bài viết kể lại vụ án hình sự đối với bị cáo G. phạm tội 'Cố ý gây thương tích' trong một xô xát tại công trình xây dựng, sau đó đã được tòa án xét xử sơ thẩm và phúc thẩm tuyên án treo nhờ sự trợ giúp pháp lý.</t>
+          <t>Công an thành phố Hải Phòng đã kịp thời ngăn chặn hai nhóm thanh thiếu niên mang theo hung khí chuẩn bị hỗn chiến và bàn giao các đối tượng liên quan để xử lý về hành vi trộm cắp tài sản.</t>
         </is>
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>Quảng Ninh</t>
+          <t>Hải Phòng</t>
         </is>
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>Khởi tố/Xét xử hình sự</t>
+          <t>Gây rối trật tự công cộng/Trộm cắp</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
@@ -839,17 +839,17 @@
     <row r="15" ht="55" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Bùi Văn Bảo</t>
+          <t>Nguyễn Văn Tình</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Bùi Văn Bảo bị Cơ quan Cảnh sát điều tra Công an tỉnh Phú Thọ ra lệnh bắt khẩn cấp về tội Chống người thi hành công vụ do không có giấy phép lái xe nhưng vẫn điều khiển xe đầu kéo vượt nhiều chốt kiểm soát và bỏ chạy 130 km.</t>
+          <t>Công an xã Ân Thi phối hợp với Công an tỉnh Hưng Yên đã bắt giữ 2 đối tượng Nguyễn Văn Tình và Nguyễn Văn Quyết có hành vi dùng dây sạc điện thoại siết cổ và kéo nhọn khống chế tài xế ô tô để cướp tài sản.</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Phú Thọ</t>
+          <t>Hưng Yên</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -859,7 +859,7 @@
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>2026-07-25
+          <t>2026-07-27
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -867,17 +867,17 @@
     <row r="16" ht="55" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>Nguyễn Thế Huynh</t>
+          <t>Lã Xuân Tuyển</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Công an tỉnh Bắc Ninh đã triệt phá đường dây sản xuất, mua bán trái phép vũ khí quân dụng (súng và đạn chì), khởi tố 16 bị can, thu giữ hàng chục nghìn viên đạn chì, hàng trăm kg chì nguyên liệu cùng nhiều tang vật liên quan.</t>
+          <t>Cơ quan Cảnh sát điều tra Công an tỉnh Ninh Bình đã khởi tố 2 bị can gồm Lã Xuân Tuyển và Phạm Công Thành về hành vi vi phạm quy định về khai thác tài nguyên, với tổng khối lượng quặng Antimon khai thác trái phép gần 1.000 tấn trị giá hơn 6,2 tỷ đồng.</t>
         </is>
       </c>
       <c r="C16" s="9" t="inlineStr">
         <is>
-          <t>Bắc Ninh</t>
+          <t>Ninh Bình</t>
         </is>
       </c>
       <c r="D16" s="10" t="inlineStr">
@@ -887,7 +887,7 @@
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>2026-07-26
+          <t>2026-07-27
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -895,27 +895,27 @@
     <row r="17" ht="55" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Công ty CP đầu tư y tế Việt Mỹ</t>
+          <t>Nguyễn Năng Mạnh</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Bộ Công an đã khởi tố vụ án, khởi tố bị can và bắt tạm giam loạt lãnh đạo Công ty CP đầu tư y tế Việt Mỹ gồm Bùi Chân Phương (nguyên Chủ tịch HĐQT), Hà Văn Nam (Giám đốc) và Trần Thị Hồng Hạnh (Kế toán) về tội Buôn lậu và Vi phạm quy định về kế toán gây hậu quả nghiêm trọng.</t>
+          <t>Chủ thương hiệu MediUSA Nguyễn Năng Mạnh cùng đồng phạm bị xét xử về các tội sản xuất, buôn bán hàng giả là thực phẩm, vi phạm quy định kế toán và đưa hối lộ. Bị cáo khai nhận đã được một cán bộ công an lộ bí mật thông tin điều tra và hướng dẫn tiêu hủy tài liệu, tẩu tán ổ cứng.</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Hải Phòng</t>
+          <t>Hà Nội</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>Khởi tố/Bắt tạm giam/Buôn lậu</t>
+          <t>Sản xuất hàng giả/Đưa hối lộ</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>2026-07-26
+          <t>2026-07-27
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -923,27 +923,27 @@
     <row r="18" ht="55" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>Lê Văn Đồng</t>
+          <t>Công ty CP đầu tư y tế Việt Mỹ</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t>Công an tỉnh Hưng Yên đã triệt phá đường dây cá độ bóng đá quy mô lớn với tổng số tiền giao dịch hơn 10,6 tỷ đồng, khởi tố và tạm giữ 10 đối tượng bao gồm Lê Văn Đồng cùng đồng phạm về tội Tổ chức đánh bạc và Đánh bạc.</t>
+          <t>Bộ Công an đã khởi tố vụ án, khởi tố bị can và bắt tạm giam loạt lãnh đạo Công ty CP đầu tư y tế Việt Mỹ gồm Bùi Chân Phương (nguyên Chủ tịch HĐQT), Hà Văn Nam (Giám đốc) và Trần Thị Hồng Hạnh (Kế toán) về tội Buôn lậu và Vi phạm quy định về kế toán gây hậu quả nghiêm trọng.</t>
         </is>
       </c>
       <c r="C18" s="9" t="inlineStr">
         <is>
-          <t>Hưng Yên</t>
+          <t>Hải Phòng</t>
         </is>
       </c>
       <c r="D18" s="10" t="inlineStr">
         <is>
-          <t>Khởi tố/Bắt tạm giam</t>
+          <t>Khởi tố/Bắt tạm giam/Buôn lậu</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>2026-07-03
+          <t>2026-07-26
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -951,17 +951,17 @@
     <row r="19" ht="55" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Đ.V.Q.</t>
+          <t>Nguyễn Thế Huynh</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>Công an thành phố Hải Phòng triệt phá đường dây cá độ bóng đá qua mạng với số tiền giao dịch hơn 11 tỷ đồng, tiến hành khởi tố và bắt tạm giam 5 đối tượng về các tội Tổ chức đánh bạc và Đánh bạc.</t>
+          <t>Công an tỉnh Bắc Ninh đã triệt phá đường dây sản xuất, mua bán trái phép vũ khí quân dụng (súng và đạn chì), khởi tố 16 bị can, thu giữ hàng chục nghìn viên đạn chì, hàng trăm kg chì nguyên liệu cùng nhiều tang vật liên quan.</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Hải Phòng</t>
+          <t>Bắc Ninh</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>2026-07-21
+          <t>2026-07-26
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -979,12 +979,12 @@
     <row r="20" ht="55" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>Chưa xác định</t>
+          <t>Công ty CP Tập đoàn Đầu tư thương mại Quang Hưng</t>
         </is>
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t>Phòng Cảnh sát giao thông Công an thành phố Hải Phòng phát hiện một thi thể nam giới khoảng 50 tuổi tại bãi bồi sông Lạch Tray và đang tiến hành xác minh danh tính.</t>
+          <t>Công an thành phố Hải Phòng đang xác minh nguồn tin về tội phạm đối với vụ việc có dấu hiệu lừa đảo chiếm đoạt tài sản liên quan đến Lưu Quang Hưng, Giám đốc Công ty CP Tập đoàn Đầu tư thương mại Quang Hưng trong các giao dịch mua bán căn hộ và đất đai.</t>
         </is>
       </c>
       <c r="C20" s="9" t="inlineStr">
@@ -994,12 +994,12 @@
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>Phát hiện tử thi</t>
+          <t>Điều tra tội phạm/Lừa đảo</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>2026-07-23
+          <t>2026-07-26
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1007,27 +1007,27 @@
     <row r="21" ht="55" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>N.T.H.</t>
+          <t>Hoàng Trọng Nguyên</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Công an xã xử phạt vi phạm hành chính 11,25 triệu đồng đối với cá nhân chia sẻ thông tin sai sự thật trên mạng xã hội về việc nữ công nhân nhiễm HIV, gây ảnh hưởng nghiêm trọng đến uy tín của Công ty TNHH Vietstar.</t>
+          <t>Hoàng Trọng Nguyên cùng nhân viên mặc áo blouse trắng, giả danh bác sĩ nha khoa có kinh nghiệm để mở phòng khám trái phép, lừa đảo chiếm đoạt tiền của nhiều bệnh nhân và bị khởi tố.</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>Hải Phòng</t>
+          <t>Lạng Sơn</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Xử phạt hành chính</t>
+          <t>Lừa dối khách hàng</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>2026-07-11
+          <t>2026-07-26
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1035,27 +1035,27 @@
     <row r="22" ht="55" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>N.V.N</t>
+          <t>Chưa xác định</t>
         </is>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t>Công an xã Hà Bắc phát hiện và xử lý đối tượng N.V.N có hành vi bẫy, nuôi nhốt trái phép chim hoang dã, tạm giữ tang vật gồm các lồng bẫy và nhiều cá thể chim.</t>
+          <t>Bão số 2 hoạt động trên Biển Đông có khả năng mạnh lên cấp 12, gây gió mạnh, sóng lớn trên biển và mưa lớn diện rộng cho khu vực Bắc Bộ và Nam Bộ, đe dọa an toàn hàng hải và nguy cơ ngập úng, sạt lở đất.</t>
         </is>
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>Hải Phòng</t>
+          <t>Quảng Ninh</t>
         </is>
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>Vi phạm quy định bảo vệ động vật hoang dã</t>
+          <t>Thiên tai/Bão lũ</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>2026-07-23
+          <t>2026-07-25
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1063,12 +1063,12 @@
     <row r="23" ht="55" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Nguyễn Văn An</t>
+          <t>Phạm Văn Chiến</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Xảy ra vụ tai nạn giao thông nghiêm trọng trên cao tốc Hà Nội - Hải Phòng giữa xe ô tô khách và xe ô tô con do bị mất lái, khiến nhiều người bị thương và 1 người tử vong.</t>
+          <t>Phòng Cảnh sát hình sự Công an thành phố Hải Phòng đã bắt giữ đối tượng Phạm Văn Chiến, nghi phạm dùng hung khí sát hại một phụ nữ tại phường Lưu Kiếm do mâu thuẫn ghen tuông tình ái.</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
@@ -1078,12 +1078,12 @@
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Tai nạn giao thông</t>
+          <t>Khởi tố/Bắt tạm giam</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>2026-07-04
+          <t>2026-07-25
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1091,27 +1091,27 @@
     <row r="24" ht="55" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>Trần Trung Đức</t>
+          <t>Thuế cơ sở 11</t>
         </is>
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>Công an tỉnh Hưng Yên thông báo tìm nhân chứng và phương tiện liên quan đến vụ tai nạn giao thông xảy ra năm 2019 tại thành phố Hưng Yên có dấu hiệu 'Vi phạm quy định về tham gia giao thông đường bộ'.</t>
+          <t>Viện Kiểm sát nhân dân khu vực 12 (Hải Phòng) có văn bản kiến nghị Thuế cơ sở 11 khắc phục việc chậm thực hiện nghĩa vụ thuế liên quan đến giao đất tái định cư, gây ảnh hưởng đến quyền lợi của một công dân cao tuổi.</t>
         </is>
       </c>
       <c r="C24" s="9" t="inlineStr">
         <is>
-          <t>Hưng Yên</t>
+          <t>Hải Phòng</t>
         </is>
       </c>
       <c r="D24" s="10" t="inlineStr">
         <is>
-          <t>Tai nạn giao thông/Truy tìm nhân chứng</t>
+          <t>Chậm thực hiện nghĩa vụ thuế</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>2026-07-24
+          <t>2026-07-25
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1119,27 +1119,27 @@
     <row r="25" ht="55" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Dương Hoài Nam</t>
+          <t>H.N.A</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>Bị cáo Dương Hoài Nam bị Tòa án nhân dân tỉnh Ninh Bình tuyên phạt án tù chung thân về tội “Mua bán trái phép chất ma túy” sau khi bị bắt quả tang vận chuyển hơn 514 gam Methamphetamine.</t>
+          <t>Lực lượng công an thành phố Hải Phòng phát hiện và xử lý nhiều nhóm thanh thiếu niên vi phạm trật tự an toàn giao thông, mang theo hung khí như kiếm dài, dao, tuýp sắt để gây rối trật tự công cộng. Trong 6 tháng đầu năm 2026, cơ quan điều tra đã khởi tố 23 vụ với 215 bị can liên quan đến tội phạm đường phố.</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>Ninh Bình</t>
+          <t>Hải Phòng</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Khởi tố/Bắt tạm giam</t>
+          <t>Khởi tố/Gây rối trật tự công cộng</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>2026-07-18
+          <t>2026-07-25
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1147,27 +1147,27 @@
     <row r="26" ht="55" customHeight="1">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>Nguyễn Văn Hào</t>
+          <t>Bùi Văn Bảo</t>
         </is>
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>Công an tỉnh Ninh Bình đã triệt phá đường dây cá độ bóng đá trên không gian mạng với số tiền giao dịch hơn 900 tỷ đồng, tạm giữ hình sự 6 đối tượng trong đó có Nguyễn Văn Hào và Phạm Xuân Thủy cầm đầu.</t>
+          <t>Bùi Văn Bảo không có giấy phép lái xe, điều khiển xe đầu kéo cơi nới thành thùng, không chấp hành hiệu lệnh dừng xe, đâm đổ các chốt kiểm soát và bỏ chạy 130 km trước khi bị bắt khẩn cấp.</t>
         </is>
       </c>
       <c r="C26" s="9" t="inlineStr">
         <is>
-          <t>Ninh Bình</t>
+          <t>Phú Thọ</t>
         </is>
       </c>
       <c r="D26" s="10" t="inlineStr">
         <is>
-          <t>Khởi tố/Bắt tạm giam</t>
+          <t>Chống người thi hành công vụ</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>2026-07-06
+          <t>2026-07-25
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1175,27 +1175,27 @@
     <row r="27" ht="55" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Tống Thị Hồng</t>
+          <t>Phòng khám Đa khoa Y học Nghệ An</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>Tòa án nhân dân tỉnh Ninh Bình đã xét xử và tuyên phạt tổng mức án 40 năm tù đối với 3 bị cáo gồm Tống Thị Hồng, Đinh Thị Hiên và Nguyễn Thị Thu Hoài về tội “Mua bán người dưới 16 tuổi” do thực hiện tiếp nhận và chuyển giao 8 trẻ sơ sinh trái pháp luật.</t>
+          <t>Phòng khám Đa khoa Y học Nghệ An bị phản ánh sử dụng chiêu trò quảng cáo giá rẻ, dọa dẫm bệnh nhân mắc bệnh nặng ngay trên bàn mổ để ép buộc làm thêm dịch vụ và nâng khống chi phí điều trị gấp nhiều lần.</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>Ninh Bình</t>
+          <t>Nghệ An</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>Khởi tố/Bắt tạm giam</t>
+          <t>Lừa đảo/Gian lận y tế</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>2026-07-17
+          <t>2026-07-25
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1203,27 +1203,27 @@
     <row r="28" ht="55" customHeight="1">
       <c r="A28" s="8" t="inlineStr">
         <is>
-          <t>Trịnh Văn Quang</t>
+          <t>Phạm Văn Chiến</t>
         </is>
       </c>
       <c r="B28" s="8" t="inlineStr">
         <is>
-          <t>Tòa án nhân dân xét xử nhóm đối tượng gồm Trịnh Văn Quang, Đinh Văn Vượng và Nguyễn Ngọc Tuấn về tội “Lừa đảo chiếm đoạt tài sản” do giả danh nhân viên y tế bán thực phẩm chức năng kém chất lượng, chiếm đoạt hơn 111 triệu đồng của 16 bị hại.</t>
+          <t>Phạm Văn Chiến bị công an bắt giữ sau hơn 30 ngày lẩn trốn vì có hành vi dùng dao đâm tử vong chị Trần Thị Anh ở khu vực ven đường quốc lộ 10 do mâu thuẫn tình cảm.</t>
         </is>
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>Ninh Bình</t>
+          <t>Hải Phòng</t>
         </is>
       </c>
       <c r="D28" s="10" t="inlineStr">
         <is>
-          <t>Xử phạt hành chính</t>
+          <t>Khởi tố/Bắt tạm giam</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>2026-07-01
+          <t>2026-07-24
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1231,27 +1231,27 @@
     <row r="29" ht="55" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Chưa xác định</t>
+          <t>Terry Rose</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>Cơ quan Cảnh sát điều tra Công an tỉnh Bắc Ninh đã khởi tố 17 thanh, thiếu niên về tội gây rối trật tự công cộng. Do mâu thuẫn trên mạng xã hội, các đối tượng đã mang theo hung khí rượt đuổi tốc độ cao trên quốc lộ 31 dẫn đến tai nạn giao thông làm 3 người tử vong.</t>
+          <t>Một vụ án mạng tại Mỹ phát hiện sau gần 25 năm khi cảnh sát tìm thấy hài cốt của nạn nhân Kimberly Langwell được giấu dưới sàn phòng ngủ của bạn trai cũ Terry Rose. Đối tượng bị tình nghi và điều tra liên quan đến hành vi sát hại nạn nhân từ năm 1999.</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>Bắc Ninh</t>
+          <t>Beaumont</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>Khởi tố/Bắt tạm giam</t>
+          <t>Giết người/Giấu xác</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>2026-07-21
+          <t>2026-07-24
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1259,27 +1259,27 @@
     <row r="30" ht="55" customHeight="1">
       <c r="A30" s="8" t="inlineStr">
         <is>
-          <t>Nguyễn Văn Anh</t>
+          <t>Nguyễn Bá Hoàng Nam và Nguyễn Văn Quân</t>
         </is>
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
-          <t>Công an phường Bồng Lai phối hợp với Văn phòng Cảnh sát điều tra Công an tỉnh Bắc Ninh đã bắt giữ Nguyễn Văn Anh do thực hiện hàng loạt vụ trộm cắp dây cáp điện chiếu sáng với tổng trị giá hơn 150 triệu đồng.</t>
+          <t>Nguyễn Bá Hoàng Nam và Nguyễn Văn Quân lần lượt bị TAND Hà Nội tuyên án 10 năm và 5 năm tù về tội Giết người do điều khiển xe máy tốc độ cao, 'thông chốt' kiểm soát và tông trực diện vào một cán bộ cảnh sát cơ động gây thương tích nặng 73%.</t>
         </is>
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>Bắc Ninh</t>
+          <t>Hà Nội</t>
         </is>
       </c>
       <c r="D30" s="10" t="inlineStr">
         <is>
-          <t>Khởi tố/Bắt tạm giam</t>
+          <t>Chống người thi hành công vụ/Giết người</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>2026-07-21
+          <t>2026-07-24
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1287,27 +1287,27 @@
     <row r="31" ht="55" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>Nguyễn Văn Minh</t>
+          <t>Nguyễn Chí Việt</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>Phòng Cảnh sát thi hành án hình sự và hỗ trợ tư pháp Công an tỉnh Bắc Ninh đã bắt giữ đối tượng truy nã Nguyễn Văn Minh về tội 'Gây rối trật tự công cộng' sau khi đối tượng trốn sang Campuchia và tìm cách che giấu nhân thân khi về nước.</t>
+          <t>Nguyễn Chí Việt và đồng phạm bị TAND TP HCM tuyên phạt án tử hình do tham gia đường dây vận chuyển, cất giấu trái phép hơn 25,5 kg ma túy ngụy trang trong giỏ quà Tết.</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>Bắc Ninh</t>
+          <t>Hồ Chí Minh</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>Truy nã/Trốn thi hành án</t>
+          <t>Khởi tố/Bắt tạm giam</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>2026-07-22
+          <t>2026-07-24
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1315,27 +1315,27 @@
     <row r="32" ht="55" customHeight="1">
       <c r="A32" s="8" t="inlineStr">
         <is>
-          <t>Đinh Đức Phụng</t>
+          <t>Chưa xác định</t>
         </is>
       </c>
       <c r="B32" s="8" t="inlineStr">
         <is>
-          <t>Công an tỉnh Bắc Ninh phối hợp với Cục An ninh mạng và phòng, chống tội phạm sử dụng công nghệ cao triệt phá đường dây đánh bạc trực tuyến xuyên quốc gia quy mô lớn do Đinh Đức Phụng cầm đầu, bắt giữ 12 đối tượng với lượng tiền giao dịch lên đến hàng nghìn tỷ đồng.</t>
+          <t>Công an phường Cầu Ông Lãnh đang xác minh vụ việc một cô gái có hành vi cầm gạch ném liên tục vào cửa kính một căn nhà ở trung tâm TP.HCM gây trầy xước tài sản.</t>
         </is>
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>Bắc Ninh</t>
+          <t>Hồ Chí Minh</t>
         </is>
       </c>
       <c r="D32" s="10" t="inlineStr">
         <is>
-          <t>Khởi tố/Bắt tạm giam</t>
+          <t>Hủy hoại tài sản/Gây rối trật tự</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>2026-07-15
+          <t>2026-07-24
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1343,27 +1343,27 @@
     <row r="33" ht="55" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>Công ty Cổ phần sản xuất phân bón Hà Bắc</t>
+          <t>Trần Trung Đức</t>
         </is>
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>Công an tỉnh Bắc Ninh đã khởi tố bị can và bắt tạm giam L.Q.N, Chủ tịch HĐQT Công ty Cổ phần sản xuất phân bón Hà Bắc, về hành vi sản xuất, buôn bán 65 tấn phân bón giả trị giá hơn 1 tỷ đồng.</t>
+          <t>Công an tỉnh Hưng Yên thông báo tìm nhân chứng và phương tiện liên quan đến vụ tai nạn giao thông xảy ra năm 2019 tại thành phố Hưng Yên có dấu hiệu 'Vi phạm quy định về tham gia giao thông đường bộ'.</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>Bắc Ninh</t>
+          <t>Hưng Yên</t>
         </is>
       </c>
       <c r="D33" s="6" t="inlineStr">
         <is>
-          <t>Khởi tố/Bắt tạm giam</t>
+          <t>Tai nạn giao thông/Truy tìm nhân chứng</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>2026-07-21
+          <t>2026-07-24
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1371,17 +1371,17 @@
     <row r="34" ht="55" customHeight="1">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t>Nguyễn Long Cảnh</t>
+          <t>Võ Thị Phương Anh</t>
         </is>
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>Cơ quan Cảnh sát điều tra Công an tỉnh Bắc Ninh ra quyết định tạm giữ đối với Nguyễn Long Cảnh để điều tra về hành vi trộm cắp tài sản sau khi đột nhập vào nhà dân lấy trộm điện thoại.</t>
+          <t>Võ Thị Phương Anh bị Công an tỉnh Hà Tĩnh bắt tạm giam về tội Lừa đảo chiếm đoạt tài sản sau khi tiếp tục dùng thủ đoạn gian dối nhận tiền chạy du học, xuất khẩu lao động để chiếm đoạt gần 700 triệu đồng trong thời gian được hoãn thi hành án.</t>
         </is>
       </c>
       <c r="C34" s="9" t="inlineStr">
         <is>
-          <t>Bắc Ninh</t>
+          <t>Hà Tĩnh</t>
         </is>
       </c>
       <c r="D34" s="10" t="inlineStr">
@@ -1391,7 +1391,7 @@
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>2026-07-20
+          <t>2026-07-23
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1399,27 +1399,27 @@
     <row r="35" ht="55" customHeight="1">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>Lê Trung Hiếu</t>
+          <t>Mai Thị Bích Vân</t>
         </is>
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>Cơ quan Cảnh sát điều tra Công an tỉnh Thái Nguyên đã khởi tố vụ án, khởi tố bị can đối với Lê Trung Hiếu cùng các đồng phạm về tội sử dụng mạng máy tính, mạng viễn thông, phương tiện điện tử thực hiện hành vi chiếm đoạt tài sản và vi phạm quy định về kinh doanh theo phương thức đa cấp thông qua đường dây tiền ảo Canvanex với hơn 3.000 bị hại và tổng số tiền 100 tỷ đồng.</t>
+          <t>Bà Mai Thị Bích Vân bị TAND khu vực 4 Hà Nội xét xử về tội Cố ý làm hư hỏng tài sản do dùng chìa khóa cào xước ô tô Mercedes đỗ chắn cổng nhà mình, gây thiệt hại tài sản.</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>Bắc Ninh</t>
+          <t>Hà Nội</t>
         </is>
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>Khởi tố/Bắt tạm giam</t>
+          <t>Xử phạt hành chính/Tố tụng hình sự</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>2026-07-19
+          <t>2026-07-23
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1427,17 +1427,17 @@
     <row r="36" ht="55" customHeight="1">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t>Lưu Văn Từ</t>
+          <t>Hà Văn Hiếu</t>
         </is>
       </c>
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>Cơ quan Cảnh sát điều tra Công an tỉnh Bắc Ninh đã ra quyết định khởi tố 21 bị can (trong đó có Lưu Văn Từ tội tổ chức đánh bạc) liên quan đến ổ nhóm đánh bạc dưới hình thức xóc đĩa tại xã Lục Ngạn.</t>
+          <t>Công an tỉnh Lai Châu phối hợp với Công an Lào triệt phá đường dây lừa đảo xuyên biên giới do Hà Văn Hiếu cầm đầu. Nhóm này giả nhân viên bảo hiểm gọi điện hướng dẫn nạn nhân quét mã QR giả để chiếm đoạt hơn 5 tỷ đồng của hơn 1.000 bị hại.</t>
         </is>
       </c>
       <c r="C36" s="9" t="inlineStr">
         <is>
-          <t>Bắc Ninh</t>
+          <t>Lai Châu</t>
         </is>
       </c>
       <c r="D36" s="10" t="inlineStr">
@@ -1447,7 +1447,7 @@
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>2026-07-17
+          <t>2026-07-23
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1455,22 +1455,22 @@
     <row r="37" ht="55" customHeight="1">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>Công ty Cổ phần Thái Hòa</t>
+          <t>Barry Minkow</t>
         </is>
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>Công an tỉnh Quảng Ninh phát hiện nhiều cơ sở giết mổ gia súc hoạt động không phép, vi phạm quy định về an toàn thực phẩm, bảo vệ môi trường và xả nước thải vượt quy chuẩn kỹ thuật, trong đó có cơ sở của Công ty Cổ phần Thái Hòa.</t>
+          <t>Bài viết kể lại vụ án lừa đảo lịch sử tại Mỹ của Barry Minkow, người sáng lập công ty ZZZZ Best, thông qua việc làm giả các hợp đồng phục hồi tài sản, báo cáo doanh thu và tài liệu thuế để chiếm đoạt hàng triệu USD tiền vay và phát hành cổ phiếu.</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Quảng Ninh</t>
+          <t>Los Angeles</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>Vi phạm môi trường/An toàn thực phẩm</t>
+          <t>Gian lận tài chính/Lừa đảo</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
@@ -1483,27 +1483,27 @@
     <row r="38" ht="55" customHeight="1">
       <c r="A38" s="8" t="inlineStr">
         <is>
-          <t>Giang Quế Dinh</t>
+          <t>Phạm Văn Chiến</t>
         </is>
       </c>
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>Cơ quan Cảnh sát điều tra Công an tỉnh Thanh Hóa đã khởi tố 12 người về tội 'Sản xuất, buôn bán hàng giả' và 1 người về tội 'Trốn thuế' liên quan đến đường dây nhập khẩu hương liệu để sản xuất, tiêu thụ nước hoa giả các thương hiệu nổi tiếng.</t>
+          <t>Phạm Văn Chiến bị cơ quan công an truy tìm do nghi ngờ sát hại chị Trần Thị Ánh bằng cách đâm nhiều nhát tại khu vực ven đường ở Hải Phòng, nghi do mâu thuẫn tình cảm.</t>
         </is>
       </c>
       <c r="C38" s="9" t="inlineStr">
         <is>
-          <t>Thanh Hóa</t>
+          <t>Hải Phòng</t>
         </is>
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
-          <t>Khởi tố/Sản xuất hàng giả/Trốn thuế</t>
+          <t>Truy nã/Giết người</t>
         </is>
       </c>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t>2026-07-22
+          <t>2026-07-23
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1511,27 +1511,27 @@
     <row r="39" ht="55" customHeight="1">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>Chưa xác định</t>
+          <t>Công ty Cổ phần Thái Hòa</t>
         </is>
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>Công an phường Cầu Ông Lãnh đang xác minh vụ việc một cô gái có hành vi cầm gạch ném liên tục vào cửa kính một căn nhà ở trung tâm TP.HCM gây trầy xước tài sản.</t>
+          <t>Công an tỉnh Quảng Ninh phát hiện nhiều cơ sở giết mổ gia súc hoạt động không phép, vi phạm quy định về an toàn thực phẩm, bảo vệ môi trường và xả nước thải vượt quy chuẩn kỹ thuật, trong đó có cơ sở của Công ty Cổ phần Thái Hòa.</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Hồ Chí Minh</t>
+          <t>Quảng Ninh</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>Hủy hoại tài sản/Gây rối trật tự</t>
+          <t>Vi phạm môi trường/An toàn thực phẩm</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>2026-07-24
+          <t>2026-07-23
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1539,27 +1539,27 @@
     <row r="40" ht="55" customHeight="1">
       <c r="A40" s="8" t="inlineStr">
         <is>
-          <t>Nguyễn Chí Việt</t>
+          <t>N.V.N</t>
         </is>
       </c>
       <c r="B40" s="8" t="inlineStr">
         <is>
-          <t>Nguyễn Chí Việt và đồng phạm bị TAND TP HCM tuyên phạt án tử hình do tham gia đường dây vận chuyển, cất giấu trái phép hơn 25,5 kg ma túy ngụy trang trong giỏ quà Tết.</t>
+          <t>Công an xã Hà Bắc phát hiện và xử lý đối tượng N.V.N có hành vi bẫy, nuôi nhốt trái phép chim hoang dã, tạm giữ tang vật gồm các lồng bẫy và nhiều cá thể chim.</t>
         </is>
       </c>
       <c r="C40" s="9" t="inlineStr">
         <is>
-          <t>Hồ Chí Minh</t>
+          <t>Hải Phòng</t>
         </is>
       </c>
       <c r="D40" s="10" t="inlineStr">
         <is>
-          <t>Khởi tố/Bắt tạm giam</t>
+          <t>Vi phạm quy định bảo vệ động vật hoang dã</t>
         </is>
       </c>
       <c r="E40" s="7" t="inlineStr">
         <is>
-          <t>2026-07-24
+          <t>2026-07-23
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1567,27 +1567,27 @@
     <row r="41" ht="55" customHeight="1">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>Phạm Thị Huyền</t>
+          <t>Chưa xác định</t>
         </is>
       </c>
       <c r="B41" s="4" t="inlineStr">
         <is>
-          <t>Phạm Thị Huyền bị Công an tỉnh Bắc Ninh khởi tố, cấm đi khỏi nơi cư trú về tội Xâm phạm quyền sở hữu công nghiệp khi bày bán gần 4 tỷ đồng trang sức giả mạo các nhãn hiệu nổi tiếng.</t>
+          <t>Phòng Cảnh sát giao thông Công an thành phố Hải Phòng phát hiện một thi thể nam giới khoảng 50 tuổi tại bãi bồi sông Lạch Tray và đang tiến hành xác minh danh tính.</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Bắc Ninh</t>
+          <t>Hải Phòng</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>Khởi tố/Bắt tạm giam</t>
+          <t>Phát hiện tử thi</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>2026-07-22
+          <t>2026-07-23
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1595,22 +1595,22 @@
     <row r="42" ht="55" customHeight="1">
       <c r="A42" s="8" t="inlineStr">
         <is>
-          <t>Phạm Văn Chiến</t>
+          <t>Lê Duy Khánh</t>
         </is>
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t>Phạm Văn Chiến bị cơ quan công an truy tìm do nghi ngờ sát hại chị Trần Thị Ánh bằng cách đâm nhiều nhát tại khu vực ven đường ở Hải Phòng, nghi do mâu thuẫn tình cảm.</t>
+          <t>Lê Duy Khánh bị TAND TP HCM tuyên phạt 4 năm tù vì hành vi 6 lần lẻn vào căn hộ hàng xóm trộm cắp tài sản gồm túi xách hàng hiệu, đồng hồ, nữ trang tổng trị giá gần 200 triệu đồng và phải bồi thường thiệt hại.</t>
         </is>
       </c>
       <c r="C42" s="9" t="inlineStr">
         <is>
-          <t>Hải Phòng</t>
+          <t>Hồ Chí Minh</t>
         </is>
       </c>
       <c r="D42" s="10" t="inlineStr">
         <is>
-          <t>Truy nã/Giết người</t>
+          <t>Trộm cắp tài sản</t>
         </is>
       </c>
       <c r="E42" s="7" t="inlineStr">
@@ -1623,27 +1623,27 @@
     <row r="43" ht="55" customHeight="1">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>Neil Lewis</t>
+          <t>Nữ giáo sư Trường Dược Đại học Sungkyunkwan</t>
         </is>
       </c>
       <c r="B43" s="4" t="inlineStr">
         <is>
-          <t>Thợ sửa ôtô Neil Lewis đã nhận tội tại tòa vì hành vi cố ý cấp giấy chứng nhận kiểm định an toàn giả cho một chiếc xe ô tô bị lỗi nặng hệ thống phanh, dây an toàn và túi khí, dẫn đến tai nạn giao thông khiến 3 người tử vong.</t>
+          <t>Một nữ giảng viên đại học tại Hàn Quốc bị kết tội Cản trở hoạt động của tổ chức vì ép sinh viên làm nghiên cứu và viết luận hộ con gái, giúp con vào trường đại học top đầu. Tòa án đã tuyên phạt bà 3 năm 6 tháng tù giam.</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Nước ngoài</t>
+          <t>Seoul</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>Vi phạm quy định an toàn/Gian lận</t>
+          <t>Khởi tố/Bắt tạm giam</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>2026-07-24
+          <t>2026-07-22
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1651,27 +1651,27 @@
     <row r="44" ht="55" customHeight="1">
       <c r="A44" s="8" t="inlineStr">
         <is>
-          <t>Lê Duy Khánh</t>
+          <t>Phạm Thị Huyền</t>
         </is>
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>Lê Duy Khánh bị TAND TP HCM tuyên phạt phúc thẩm mức án 4 năm tù về tội Trộm cắp tài sản do có hành vi 6 lần lẻn vào nhà hàng xom trộm cắp túi xách hàng hiệu, nữ trang trị giá gần 200 triệu đồng và phải bồi thường theo quy định.</t>
+          <t>Phạm Thị Huyền bị Công an tỉnh Bắc Ninh khởi tố, cấm đi khỏi nơi cư trú về tội Xâm phạm quyền sở hữu công nghiệp khi bày bán gần 4 tỷ đồng trang sức giả mạo các nhãn hiệu nổi tiếng.</t>
         </is>
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>Hồ Chí Minh</t>
+          <t>Bắc Ninh</t>
         </is>
       </c>
       <c r="D44" s="10" t="inlineStr">
         <is>
-          <t>Trộm cắp tài sản</t>
+          <t>Khởi tố/Bắt tạm giam</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>2026-07-23
+          <t>2026-07-22
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1679,27 +1679,27 @@
     <row r="45" ht="55" customHeight="1">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>Nguyễn Bá Hoàng Nam và Nguyễn Văn Quân</t>
+          <t>Giang Quế Dinh</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
         <is>
-          <t>Nguyễn Bá Hoàng Nam và Nguyễn Văn Quân lần lượt bị TAND Hà Nội tuyên án 10 năm và 5 năm tù về tội Giết người do điều khiển xe máy tốc độ cao, 'thông chốt' kiểm soát và tông trực diện vào một cán bộ cảnh sát cơ động gây thương tích nặng 73%.</t>
+          <t>Cơ quan Cảnh sát điều tra Công an tỉnh Thanh Hóa đã khởi tố 12 người về tội 'Sản xuất, buôn bán hàng giả' và 1 người về tội 'Trốn thuế' liên quan đến đường dây nhập khẩu hương liệu để sản xuất, tiêu thụ nước hoa giả các thương hiệu nổi tiếng.</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Hà Nội</t>
+          <t>Thanh Hóa</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>Chống người thi hành công vụ/Giết người</t>
+          <t>Khởi tố/Sản xuất hàng giả/Trốn thuế</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>2026-07-24
+          <t>2026-07-22
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1707,22 +1707,22 @@
     <row r="46" ht="55" customHeight="1">
       <c r="A46" s="8" t="inlineStr">
         <is>
-          <t>Nữ giáo sư Trường Dược Đại học Sungkyunkwan</t>
+          <t>Nguyễn Văn Minh</t>
         </is>
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>Một nữ giảng viên đại học tại Hàn Quốc bị kết tội Cản trở hoạt động của tổ chức vì ép sinh viên làm nghiên cứu và viết luận hộ con gái, giúp con vào trường đại học top đầu. Tòa án đã tuyên phạt bà 3 năm 6 tháng tù giam.</t>
+          <t>Phòng Cảnh sát thi hành án hình sự và hỗ trợ tư pháp Công an tỉnh Bắc Ninh đã bắt giữ đối tượng truy nã Nguyễn Văn Minh về tội 'Gây rối trật tự công cộng' sau khi đối tượng trốn sang Campuchia và tìm cách che giấu nhân thân khi về nước.</t>
         </is>
       </c>
       <c r="C46" s="9" t="inlineStr">
         <is>
-          <t>Seoul</t>
+          <t>Bắc Ninh</t>
         </is>
       </c>
       <c r="D46" s="10" t="inlineStr">
         <is>
-          <t>Khởi tố/Bắt tạm giam</t>
+          <t>Truy nã/Trốn thi hành án</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
@@ -1735,27 +1735,27 @@
     <row r="47" ht="55" customHeight="1">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>Barry Minkow</t>
+          <t>Công ty Cổ phần sản xuất phân bón Hà Bắc</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Bài viết kể lại vụ án lừa đảo lịch sử tại Mỹ của Barry Minkow, người sáng lập công ty ZZZZ Best, thông qua việc làm giả các hợp đồng phục hồi tài sản, báo cáo doanh thu và tài liệu thuế để chiếm đoạt hàng triệu USD tiền vay và phát hành cổ phiếu.</t>
+          <t>Công an tỉnh Bắc Ninh đã khởi tố bị can và bắt tạm giam L.Q.N, Chủ tịch HĐQT Công ty Cổ phần sản xuất phân bón Hà Bắc, về hành vi sản xuất, buôn bán 65 tấn phân bón giả trị giá hơn 1 tỷ đồng.</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Los Angeles</t>
+          <t>Bắc Ninh</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>Gian lận tài chính/Lừa đảo</t>
+          <t>Khởi tố/Bắt tạm giam</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>2026-07-23
+          <t>2026-07-21
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1763,17 +1763,17 @@
     <row r="48" ht="55" customHeight="1">
       <c r="A48" s="8" t="inlineStr">
         <is>
-          <t>Hà Văn Hiếu</t>
+          <t>Nguyễn Văn Anh</t>
         </is>
       </c>
       <c r="B48" s="8" t="inlineStr">
         <is>
-          <t>Công an tỉnh Lai Châu phối hợp với Công an Lào triệt phá đường dây lừa đảo xuyên biên giới do Hà Văn Hiếu cầm đầu. Nhóm này giả nhân viên bảo hiểm gọi điện hướng dẫn nạn nhân quét mã QR giả để chiếm đoạt hơn 5 tỷ đồng của hơn 1.000 bị hại.</t>
+          <t>Công an phường Bồng Lai phối hợp với Văn phòng Cảnh sát điều tra Công an tỉnh Bắc Ninh đã bắt giữ Nguyễn Văn Anh do thực hiện hàng loạt vụ trộm cắp dây cáp điện chiếu sáng với tổng trị giá hơn 150 triệu đồng.</t>
         </is>
       </c>
       <c r="C48" s="9" t="inlineStr">
         <is>
-          <t>Lai Châu</t>
+          <t>Bắc Ninh</t>
         </is>
       </c>
       <c r="D48" s="10" t="inlineStr">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>2026-07-23
+          <t>2026-07-21
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1791,27 +1791,27 @@
     <row r="49" ht="55" customHeight="1">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>Terry Rose</t>
+          <t>Chưa xác định</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>Một vụ án mạng tại Mỹ phát hiện sau gần 25 năm khi cảnh sát tìm thấy hài cốt của nạn nhân Kimberly Langwell được giấu dưới sàn phòng ngủ của bạn trai cũ Terry Rose. Đối tượng bị tình nghi và điều tra liên quan đến hành vi sát hại nạn nhân từ năm 1999.</t>
+          <t>Cơ quan Cảnh sát điều tra Công an tỉnh Bắc Ninh đã khởi tố 17 thanh, thiếu niên về tội gây rối trật tự công cộng. Do mâu thuẫn trên mạng xã hội, các đối tượng đã mang theo hung khí rượt đuổi tốc độ cao trên quốc lộ 31 dẫn đến tai nạn giao thông làm 3 người tử vong.</t>
         </is>
       </c>
       <c r="C49" s="5" t="inlineStr">
         <is>
-          <t>Beaumont</t>
+          <t>Bắc Ninh</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>Giết người/Giấu xác</t>
+          <t>Khởi tố/Bắt tạm giam</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>2026-07-24
+          <t>2026-07-21
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1819,12 +1819,12 @@
     <row r="50" ht="55" customHeight="1">
       <c r="A50" s="8" t="inlineStr">
         <is>
-          <t>Phạm Văn Chiến</t>
+          <t>Đ.V.Q.</t>
         </is>
       </c>
       <c r="B50" s="8" t="inlineStr">
         <is>
-          <t>Phạm Văn Chiến bị công an bắt giữ sau hơn 30 ngày lẩn trốn vì có hành vi dùng dao đâm tử vong chị Trần Thị Anh ở khu vực ven đường quốc lộ 10 do mâu thuẫn tình cảm.</t>
+          <t>Công an thành phố Hải Phòng triệt phá đường dây cá độ bóng đá qua mạng với số tiền giao dịch hơn 11 tỷ đồng, tiến hành khởi tố và bắt tạm giam 5 đối tượng về các tội Tổ chức đánh bạc và Đánh bạc.</t>
         </is>
       </c>
       <c r="C50" s="9" t="inlineStr">
@@ -1839,7 +1839,7 @@
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>2026-07-24
+          <t>2026-07-21
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1847,27 +1847,27 @@
     <row r="51" ht="55" customHeight="1">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>Mai Thị Bích Vân</t>
+          <t>Neil Lewis</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>Bà Mai Thị Bích Vân bị TAND khu vực 4 Hà Nội xét xử về tội Cố ý làm hư hỏng tài sản do dùng chìa khóa cào xước ô tô Mercedes đỗ chắn cổng nhà mình, gây thiệt hại tài sản.</t>
+          <t>Thợ sửa ôtô Neil Lewis đã cố ý cấp giấy chứng nhận kiểm định an toàn giả cho chiếc xe Volkswagen Tiguan vốn bị lỗi nghiêm trọng về dây an toàn và túi khí. Hậu quả khiến xe mất lái vào tháng 3/2023 làm 3 người tử vong và 2 người bị thương nặng; đối tượng đã nhận tội gian lận trước tòa.</t>
         </is>
       </c>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>Hà Nội</t>
+          <t>Nước ngoài</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>Xử phạt hành chính/Tố tụng hình sự</t>
+          <t>Gian lận/Vi phạm quy định an toàn</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>2026-07-23
+          <t>2026-07-21
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1875,17 +1875,17 @@
     <row r="52" ht="55" customHeight="1">
       <c r="A52" s="8" t="inlineStr">
         <is>
-          <t>Võ Thị Phương Anh</t>
+          <t>Nguyễn Long Cảnh</t>
         </is>
       </c>
       <c r="B52" s="8" t="inlineStr">
         <is>
-          <t>Võ Thị Phương Anh bị Công an tỉnh Hà Tĩnh bắt tạm giam về tội Lừa đảo chiếm đoạt tài sản sau khi tiếp tục dùng thủ đoạn gian dối nhận tiền chạy du học, xuất khẩu lao động để chiếm đoạt gần 700 triệu đồng trong thời gian được hoãn thi hành án.</t>
+          <t>Cơ quan Cảnh sát điều tra Công an tỉnh Bắc Ninh ra quyết định tạm giữ đối với Nguyễn Long Cảnh để điều tra về hành vi trộm cắp tài sản sau khi đột nhập vào nhà dân lấy trộm điện thoại.</t>
         </is>
       </c>
       <c r="C52" s="9" t="inlineStr">
         <is>
-          <t>Hà Tĩnh</t>
+          <t>Bắc Ninh</t>
         </is>
       </c>
       <c r="D52" s="10" t="inlineStr">
@@ -1895,7 +1895,7 @@
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>2026-07-23
+          <t>2026-07-20
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1903,12 +1903,12 @@
     <row r="53" ht="55" customHeight="1">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>Bệnh viện Đa khoa Bắc Ninh số 2</t>
+          <t>Lê Trung Hiếu</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>Bệnh viện Đa khoa Bắc Ninh số 2 đã tạm đình chỉ công tác 2 nhân viên thu vé xe sau phản ánh của bạn đọc. Ngoài ra, bài báo tổng hợp các phản ánh về vi phạm đất bãi sông, ô nhiễm môi trường và trật tự đô thị trên địa bàn tỉnh.</t>
+          <t>Cơ quan Cảnh sát điều tra Công an tỉnh Thái Nguyên đã khởi tố vụ án, khởi tố bị can đối với Lê Trung Hiếu cùng các đồng phạm về tội sử dụng mạng máy tính, mạng viễn thông, phương tiện điện tử thực hiện hành vi chiếm đoạt tài sản và vi phạm quy định về kinh doanh theo phương thức đa cấp thông qua đường dây tiền ảo Canvanex với hơn 3.000 bị hại và tổng số tiền 100 tỷ đồng.</t>
         </is>
       </c>
       <c r="C53" s="5" t="inlineStr">
@@ -1918,12 +1918,12 @@
       </c>
       <c r="D53" s="6" t="inlineStr">
         <is>
-          <t>Vi phạm nội quy/Xử lý nhân sự</t>
+          <t>Khởi tố/Bắt tạm giam</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>2026-07-02
+          <t>2026-07-19
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1931,17 +1931,17 @@
     <row r="54" ht="55" customHeight="1">
       <c r="A54" s="8" t="inlineStr">
         <is>
-          <t>Nguyễn Văn Mong</t>
+          <t>Dương Hoài Nam</t>
         </is>
       </c>
       <c r="B54" s="8" t="inlineStr">
         <is>
-          <t>Tòa án nhân dân tỉnh Bắc Ninh tuyên phạt bị cáo Nguyễn Văn Mong tổng mức án 18 năm tù về tội mua bán trái phép chất ma túy với vai trò cầm đầu ổ nhóm bán lẻ. Các đồng phạm khác cũng bị tuyên án từ 5 năm 6 tháng đến 8 năm 6 tháng tù.</t>
+          <t>Bị cáo Dương Hoài Nam bị Tòa án nhân dân tỉnh Ninh Bình tuyên phạt án tù chung thân về tội “Mua bán trái phép chất ma túy” sau khi bị bắt quả tang vận chuyển hơn 514 gam Methamphetamine.</t>
         </is>
       </c>
       <c r="C54" s="9" t="inlineStr">
         <is>
-          <t>Bắc Ninh</t>
+          <t>Ninh Bình</t>
         </is>
       </c>
       <c r="D54" s="10" t="inlineStr">
@@ -1951,7 +1951,7 @@
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>2026-07-28
+          <t>2026-07-18
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1959,27 +1959,27 @@
     <row r="55" ht="55" customHeight="1">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>Chưa xác định</t>
+          <t>Lưu Văn Từ</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>Cơ quan Cảnh sát điều tra Công an tỉnh Quảng Ninh đã ban hành kết luận điều tra, đề nghị truy tố 1 đối tượng về hành vi 'Lừa đảo chiếm đoạt tài sản' liên quan đến việc sử dụng Giấy chứng nhận quyền sử dụng đất giả.</t>
+          <t>Cơ quan Cảnh sát điều tra Công an tỉnh Bắc Ninh đã ra quyết định khởi tố 21 bị can (trong đó có Lưu Văn Từ tội tổ chức đánh bạc) liên quan đến ổ nhóm đánh bạc dưới hình thức xóc đĩa tại xã Lục Ngạn.</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>Quảng Ninh</t>
+          <t>Bắc Ninh</t>
         </is>
       </c>
       <c r="D55" s="6" t="inlineStr">
         <is>
-          <t>Khởi tố/Đề nghị truy tố</t>
+          <t>Khởi tố/Bắt tạm giam</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>2026-05-21
+          <t>2026-07-17
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -1987,27 +1987,27 @@
     <row r="56" ht="55" customHeight="1">
       <c r="A56" s="8" t="inlineStr">
         <is>
-          <t>Công ty MediUSA</t>
+          <t>Tống Thị Hồng</t>
         </is>
       </c>
       <c r="B56" s="8" t="inlineStr">
         <is>
-          <t>TAND Hà Nội xét xử vụ án sản xuất 88 dòng thực phẩm chức năng giả liên quan đến cựu CEO Nguyễn Năng Mạnh của Công ty MediUSA. Hai cựu cán bộ thuộc Cục Giám sát quản lý về Hải quan bị truy tố tội Nhận hối lộ vì đã nhận 1,5 tỷ đồng để giúp công ty này thông quan trái phép lô nguyên liệu trị giá 20 tỷ đồng.</t>
+          <t>Tòa án nhân dân tỉnh Ninh Bình đã xét xử và tuyên phạt tổng mức án 40 năm tù đối với 3 bị cáo gồm Tống Thị Hồng, Đinh Thị Hiên và Nguyễn Thị Thu Hoài về tội “Mua bán người dưới 16 tuổi” do thực hiện tiếp nhận và chuyển giao 8 trẻ sơ sinh trái pháp luật.</t>
         </is>
       </c>
       <c r="C56" s="9" t="inlineStr">
         <is>
-          <t>Hà Nội</t>
+          <t>Ninh Bình</t>
         </is>
       </c>
       <c r="D56" s="10" t="inlineStr">
         <is>
-          <t>Nhận hối lộ/Sản xuất hàng giả</t>
+          <t>Khởi tố/Bắt tạm giam</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>2026-07-28
+          <t>2026-07-17
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -2015,27 +2015,279 @@
     <row r="57" ht="55" customHeight="1">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>Hứa Văn Xương</t>
+          <t>Đinh Đức Phụng</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>Lực lượng chức năng tại Hưng Yên đã bắt quả tang đối tượng Hứa Văn Xương đang vận chuyển trái phép 30.000 viên ma túy tổng hợp có khối lượng gần 2,8kg tại khu vực Trạm thu phí cầu Thái Hà.</t>
+          <t>Công an tỉnh Bắc Ninh phối hợp với Cục An ninh mạng và phòng, chống tội phạm sử dụng công nghệ cao triệt phá đường dây đánh bạc trực tuyến xuyên quốc gia quy mô lớn do Đinh Đức Phụng cầm đầu, bắt giữ 12 đối tượng với lượng tiền giao dịch lên đến hàng nghìn tỷ đồng.</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
+          <t>Bắc Ninh</t>
+        </is>
+      </c>
+      <c r="D57" s="6" t="inlineStr">
+        <is>
+          <t>Khởi tố/Bắt tạm giam</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-15
+(Xem bài gốc)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="55" customHeight="1">
+      <c r="A58" s="8" t="inlineStr">
+        <is>
+          <t>N.T.H.</t>
+        </is>
+      </c>
+      <c r="B58" s="8" t="inlineStr">
+        <is>
+          <t>Công an xã xử phạt vi phạm hành chính 11,25 triệu đồng đối với cá nhân chia sẻ thông tin sai sự thật trên mạng xã hội về việc nữ công nhân nhiễm HIV, gây ảnh hưởng nghiêm trọng đến uy tín của Công ty TNHH Vietstar.</t>
+        </is>
+      </c>
+      <c r="C58" s="9" t="inlineStr">
+        <is>
+          <t>Hải Phòng</t>
+        </is>
+      </c>
+      <c r="D58" s="10" t="inlineStr">
+        <is>
+          <t>Xử phạt hành chính</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-11
+(Xem bài gốc)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="55" customHeight="1">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn Hào</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>Công an tỉnh Ninh Bình đã triệt phá đường dây cá độ bóng đá trên không gian mạng với số tiền giao dịch hơn 900 tỷ đồng, tạm giữ hình sự 6 đối tượng trong đó có Nguyễn Văn Hào và Phạm Xuân Thủy cầm đầu.</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>Ninh Bình</t>
+        </is>
+      </c>
+      <c r="D59" s="6" t="inlineStr">
+        <is>
+          <t>Khởi tố/Bắt tạm giam</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-06
+(Xem bài gốc)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="55" customHeight="1">
+      <c r="A60" s="8" t="inlineStr">
+        <is>
+          <t>Nguyễn Văn An</t>
+        </is>
+      </c>
+      <c r="B60" s="8" t="inlineStr">
+        <is>
+          <t>Xảy ra vụ tai nạn giao thông nghiêm trọng trên cao tốc Hà Nội - Hải Phòng giữa xe ô tô khách và xe ô tô con do bị mất lái, khiến nhiều người bị thương và 1 người tử vong.</t>
+        </is>
+      </c>
+      <c r="C60" s="9" t="inlineStr">
+        <is>
+          <t>Hải Phòng</t>
+        </is>
+      </c>
+      <c r="D60" s="10" t="inlineStr">
+        <is>
+          <t>Tai nạn giao thông</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-04
+(Xem bài gốc)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="55" customHeight="1">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>Lê Văn Đồng</t>
+        </is>
+      </c>
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>Công an tỉnh Hưng Yên đã triệt phá đường dây cá độ bóng đá quy mô lớn với tổng số tiền giao dịch hơn 10,6 tỷ đồng, khởi tố và tạm giữ 10 đối tượng bao gồm Lê Văn Đồng cùng đồng phạm về tội Tổ chức đánh bạc và Đánh bạc.</t>
+        </is>
+      </c>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
           <t>Hưng Yên</t>
         </is>
       </c>
-      <c r="D57" s="6" t="inlineStr">
-        <is>
-          <t>Vận chuyển ma túy trái phép</t>
-        </is>
-      </c>
-      <c r="E57" s="7" t="inlineStr">
-        <is>
-          <t>2026-07-28
+      <c r="D61" s="6" t="inlineStr">
+        <is>
+          <t>Khởi tố/Bắt tạm giam</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-03
+(Xem bài gốc)</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="55" customHeight="1">
+      <c r="A62" s="8" t="inlineStr">
+        <is>
+          <t>Bệnh viện Đa khoa Bắc Ninh số 2</t>
+        </is>
+      </c>
+      <c r="B62" s="8" t="inlineStr">
+        <is>
+          <t>Bệnh viện Đa khoa Bắc Ninh số 2 đã tạm đình chỉ công tác 2 nhân viên thu vé xe sau phản ánh của bạn đọc. Ngoài ra, bài báo tổng hợp các phản ánh về vi phạm đất bãi sông, ô nhiễm môi trường và trật tự đô thị trên địa bàn tỉnh.</t>
+        </is>
+      </c>
+      <c r="C62" s="9" t="inlineStr">
+        <is>
+          <t>Bắc Ninh</t>
+        </is>
+      </c>
+      <c r="D62" s="10" t="inlineStr">
+        <is>
+          <t>Vi phạm nội quy/Xử lý nhân sự</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-02
+(Xem bài gốc)</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="55" customHeight="1">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>Trịnh Văn Quang</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>Tòa án nhân dân xét xử nhóm đối tượng gồm Trịnh Văn Quang, Đinh Văn Vượng và Nguyễn Ngọc Tuấn về tội “Lừa đảo chiếm đoạt tài sản” do giả danh nhân viên y tế bán thực phẩm chức năng kém chất lượng, chiếm đoạt hơn 111 triệu đồng của 16 bị hại.</t>
+        </is>
+      </c>
+      <c r="C63" s="5" t="inlineStr">
+        <is>
+          <t>Ninh Bình</t>
+        </is>
+      </c>
+      <c r="D63" s="6" t="inlineStr">
+        <is>
+          <t>Xử phạt hành chính</t>
+        </is>
+      </c>
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>2026-07-01
+(Xem bài gốc)</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="55" customHeight="1">
+      <c r="A64" s="8" t="inlineStr">
+        <is>
+          <t>Chưa xác định</t>
+        </is>
+      </c>
+      <c r="B64" s="8" t="inlineStr">
+        <is>
+          <t>Cơ quan Cảnh sát điều tra Công an tỉnh Quảng Ninh đã ban hành kết luận điều tra, đề nghị truy tố 1 đối tượng về hành vi 'Lừa đảo chiếm đoạt tài sản' liên quan đến việc sử dụng Giấy chứng nhận quyền sử dụng đất giả.</t>
+        </is>
+      </c>
+      <c r="C64" s="9" t="inlineStr">
+        <is>
+          <t>Quảng Ninh</t>
+        </is>
+      </c>
+      <c r="D64" s="10" t="inlineStr">
+        <is>
+          <t>Khởi tố/Đề nghị truy tố</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-21
+(Xem bài gốc)</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="55" customHeight="1">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>Vũ Thị Thảo</t>
+        </is>
+      </c>
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>Công an quận Lê Chân (Hải Phòng) triệt phá đường dây vận chuyển trái phép chất ma túy qua dịch vụ chuyển phát nhanh, bắt giữ 3 đối tượng gồm Vũ Thị Thảo, Nguyễn Kim Hùng và Đặng Quang Chính, thu giữ 20 gam Methamphetamine.</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="inlineStr">
+        <is>
+          <t>Hải Phòng</t>
+        </is>
+      </c>
+      <c r="D65" s="6" t="inlineStr">
+        <is>
+          <t>Khởi tố/Bắt tạm giam</t>
+        </is>
+      </c>
+      <c r="E65" s="7" t="inlineStr">
+        <is>
+          <t>2026-03-27
+(Xem bài gốc)</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="55" customHeight="1">
+      <c r="A66" s="8" t="inlineStr">
+        <is>
+          <t>Chưa xác định</t>
+        </is>
+      </c>
+      <c r="B66" s="8" t="inlineStr">
+        <is>
+          <t>Kho chứa bao bì và hàng đông lạnh rộng hơn 1.000 m2 tại xã Bình Hưng, TP HCM bốc cháy dữ dội khiến một phần mái tôn đổ sập.</t>
+        </is>
+      </c>
+      <c r="C66" s="9" t="inlineStr">
+        <is>
+          <t>Hồ Chí Minh</t>
+        </is>
+      </c>
+      <c r="D66" s="10" t="inlineStr">
+        <is>
+          <t>Hỏa hoạn/Cháy nổ</t>
+        </is>
+      </c>
+      <c r="E66" s="7" t="inlineStr">
+        <is>
+          <t>2025-07-25
 (Xem bài gốc)</t>
         </is>
       </c>
@@ -2099,6 +2351,15 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId51"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="rId62"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>